<commit_message>
Convert SWI-PRO-MET-206-002 and 206-004 to Heritage per Martabe decisions; 206 series complete
206-002: GM8902 face velocity at working sash height, average and lowest of 20 readings.
206-004: TPS cube adopted, three-point pH kept, Martabe DO method on HI9142.
201-013: cross-reference updated to 206-004 Step 3. 203-003 hearing protection approved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-206.xlsx
+++ b/docs/Register-SWI-206.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keterangan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 206'!$A$1:$Q$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 206'!$A$1:$Q$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +45,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,7 +95,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -461,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -656,17 +664,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>206-003</t>
+          <t>206-002</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-003</t>
+          <t>SWI-PRO-MET-206-002</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Balance Verification and Calibration Check</t>
+          <t>Fume Cupboard Operation, Scrubber Check and Cleaning</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -676,12 +684,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-003</t>
+          <t>JSEA-PRO-MET-206-002</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -706,23 +714,23 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Daily verification before use; full calibration at the external interval.</t>
+          <t>Every use; scrubber checked at the start of every shift; face velocity measured monthly and after any repair to the extraction fan, ductwork or scrubber.</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+          <t>Operating Anemometer GM8902 - Step 4-5, ukur di tinggi sash kerja, rata-rata dan bacaan terendah dari 20 bacaan</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -732,24 +740,24 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-003-Balance-Verification-and-Calibration-Check-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-002-Fume-Cupboard-Operation-Scrubber-Check-and-Cleaning-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>206-005</t>
+          <t>206-003</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-005</t>
+          <t>SWI-PRO-MET-206-003</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Cyanide Solution Handling and Spill Response</t>
+          <t>Balance Verification and Calibration Check</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -759,12 +767,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-005</t>
+          <t>JSEA-PRO-MET-206-003</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -789,7 +797,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Every cyanide handling task; drill at the set interval.</t>
+          <t>Daily verification before use; full calibration at the external interval.</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
@@ -815,24 +823,24 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-005-Cyanide-Solution-Handling-and-Spill-Response-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-003-Balance-Verification-and-Calibration-Check-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>206-006</t>
+          <t>206-004</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-006</t>
+          <t>SWI-PRO-MET-206-004</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Acid Spill Response and Neutralisation</t>
+          <t>pH, DO and Conductivity Meter Calibration</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -842,12 +850,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-006</t>
+          <t>JSEA-PRO-MET-206-004</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -872,23 +880,23 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Every acid handling task; drill at the set interval.</t>
+          <t>Every shift before use, and after any electrode change.</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>Tidak ada padanan</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>Final (isi tanpa tambahan)</t>
+          <t>TPS cube pH meter (kalibrasi tetap 3 titik) - Step 3-4; Operate DO Meter Portable untuk HI9142 tanpa menu Oxyguard - Step 5-6</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -898,24 +906,24 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-006-Acid-Spill-Response-and-Neutralisation-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-004-pH-DO-and-Conductivity-Meter-Calibration-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>206-007</t>
+          <t>206-005</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-007</t>
+          <t>SWI-PRO-MET-206-005</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Met Lab Waste, Residue and Effluent Disposal</t>
+          <t>Cyanide Solution Handling and Spill Response</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -930,7 +938,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-007</t>
+          <t>JSEA-PRO-MET-206-005</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -955,7 +963,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Every day, and at the end of every test.</t>
+          <t>Every cyanide handling task; drill at the set interval.</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
@@ -981,24 +989,24 @@
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-007-Met-Lab-Waste-Residue-and-Effluent-Disposal-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-005-Cyanide-Solution-Handling-and-Spill-Response-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>206-008</t>
+          <t>206-006</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-008</t>
+          <t>SWI-PRO-MET-206-006</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Glassware Cleaning and Drying</t>
+          <t>Acid Spill Response and Neutralisation</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1008,12 +1016,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-008</t>
+          <t>JSEA-PRO-MET-206-006</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1038,7 +1046,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>After every use.</t>
+          <t>Every acid handling task; drill at the set interval.</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
@@ -1064,24 +1072,24 @@
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-008-Glassware-Cleaning-and-Drying-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-006-Acid-Spill-Response-and-Neutralisation-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>206-009</t>
+          <t>206-007</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-009</t>
+          <t>SWI-PRO-MET-206-007</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Bottle Roller, Bench Mill and Agitator Operation</t>
+          <t>Met Lab Waste, Residue and Effluent Disposal</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1091,12 +1099,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-009</t>
+          <t>JSEA-PRO-MET-206-007</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1121,7 +1129,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Every testwork run using them.</t>
+          <t>Every day, and at the end of every test.</t>
         </is>
       </c>
       <c r="L8" s="2" t="n">
@@ -1147,24 +1155,24 @@
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-009-Bottle-Roller-Bench-Mill-and-Agitator-Operation-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-007-Met-Lab-Waste-Residue-and-Effluent-Disposal-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>206-010</t>
+          <t>206-008</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-010</t>
+          <t>SWI-PRO-MET-206-008</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Drying Oven and Muffle Furnace Operation</t>
+          <t>Glassware Cleaning and Drying</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1174,12 +1182,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-010</t>
+          <t>JSEA-PRO-MET-206-008</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1204,7 +1212,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Every drying and ashing operation.</t>
+          <t>After every use.</t>
         </is>
       </c>
       <c r="L9" s="2" t="n">
@@ -1230,24 +1238,24 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-010-Drying-Oven-and-Muffle-Furnace-Operation-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-008-Glassware-Cleaning-and-Drying-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>206-011</t>
+          <t>206-009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-011</t>
+          <t>SWI-PRO-MET-206-009</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Met Lab Emergency Response - Power Failure and Evacuation</t>
+          <t>Bottle Roller, Bench Mill and Agitator Operation</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1257,12 +1265,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Safety-critical</t>
+          <t>Operating</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-011</t>
+          <t>JSEA-PRO-MET-206-009</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1287,7 +1295,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>On any power failure or evacuation; drill at the set interval.</t>
+          <t>Every testwork run using them.</t>
         </is>
       </c>
       <c r="L10" s="2" t="n">
@@ -1313,24 +1321,24 @@
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-011-Met-Lab-Emergency-Response---Power-Failure-and-Evacuation-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-009-Bottle-Roller-Bench-Mill-and-Agitator-Operation-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>206-013</t>
+          <t>206-010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-013</t>
+          <t>SWI-PRO-MET-206-010</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Ductless Fume Cabinet Filter Change and Breakthrough Check</t>
+          <t>Drying Oven and Muffle Furnace Operation</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1345,7 +1353,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-013</t>
+          <t>JSEA-PRO-MET-206-010</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1370,7 +1378,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Breakthrough check monthly; filter change on indication or at the manufacturer's interval.</t>
+          <t>Every drying and ashing operation.</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
@@ -1396,24 +1404,24 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-013-Ductless-Fume-Cabinet-Filter-Change-and-Breakthrough-Check-RevA.docx</t>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-010-Drying-Oven-and-Muffle-Furnace-Operation-RevA.docx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>206-014</t>
+          <t>206-011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>SWI-PRO-MET-206-014</t>
+          <t>SWI-PRO-MET-206-011</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Met Lab Equipment Receipt, Installation and Commissioning Handover</t>
+          <t>Met Lab Emergency Response - Power Failure and Evacuation</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1423,12 +1431,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Operating</t>
+          <t>Safety-critical</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>JSEA-PRO-MET-206-014</t>
+          <t>JSEA-PRO-MET-206-011</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1453,7 +1461,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Once, at laboratory establishment; then on every new instrument.</t>
+          <t>On any power failure or evacuation; drill at the set interval.</t>
         </is>
       </c>
       <c r="L12" s="2" t="n">
@@ -1479,12 +1487,178 @@
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-011-Met-Lab-Emergency-Response---Power-Failure-and-Evacuation-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>206-013</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-206-013</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Ductless Fume Cabinet Filter Change and Breakthrough Check</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>206 Met Lab - Facility, Safety and Quality</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-206-013</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Breakthrough check monthly; filter change on indication or at the manufacturer's interval.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-206-013-Ductless-Fume-Cabinet-Filter-Change-and-Breakthrough-Check-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>206-014</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-206-014</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Met Lab Equipment Receipt, Installation and Commissioning Handover</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>206 Met Lab - Facility, Safety and Quality</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Operating</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-206-014</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Once, at laboratory establishment; then on every new instrument.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Final (isi tanpa tambahan)</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
           <t>MM-4034-033-OR-03-SWI-PRO-MET-206-014-Met-Lab-Equipment-Receipt-Installation-and-Commissioning-Handover-RevA.docx</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q12"/>
+  <autoFilter ref="A1:Q14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1495,7 +1669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1505,51 +1679,117 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>No. dokumen</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Jenis</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Isi catatan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Tidak ada draft, catatan, atau open items di seri ini.</t>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-206-002</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Fume Cupboard Operation, Scrubber Check and Cleaning</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 4 and 5 follow the Martabe work instruction Operating Anemometer GM8902 (DOC-3-MET-PMC-WIN-00130-IE, v1.0, 25/12/2024). The face velocity is measured at the marked working sash height, and the average and the lowest of 20 readings are recorded. JSEA-PRO-MET-206-002 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-206-002</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Fume Cupboard Operation, Scrubber Check and Cleaning</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Open items: (1) take the required face velocity from the Safetyflow fume cupboard specification (ILS Q0023979), or from AS/NZS 2243.8 where the specification does not give it - about 0.5 m/s average is typical and must be confirmed before use; (2) set the lowest single reading allowed; (3) confirm the monthly measurement frequency; (4) confirm the GM8902 anemometer and its calibration certificate are on site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-206-004</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>pH, DO and Conductivity Meter Calibration</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Draft for review: Steps 3 and 4 follow the Martabe work instructions pH Meter TPS Cube Calibration (DOC-3-MET-PMC-WIN-00087-IE) and Operating pH Cube Meter (DOC-3-MET-PMC-WIN-00089-IE), and Steps 5 and 6 follow Operate DO Meter Portable (DOC-3-MET-PRS-WIN-00055-IE), v1.0, 25/12/2024. The TPS pH cube meter is adopted as at Martabe. pH calibration stays at three points (pH 4, 7 and 10) with the slope and offset recorded; the Martabe two-point calibration is not used. The Martabe DO method is applied to the Hanna HI9142 meter without the Oxyguard menu steps. JSEA-PRO-MET-206-004 must be updated for the added hazards before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-206-004</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>pH, DO and Conductivity Meter Calibration</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Open items: (1) confirm the TPS pH cube meter is on site, or procure it, and add it to the asset list; (2) take the DO calibration acceptance limit in air from the HI9142 manual - the Martabe value of 6 to 8 has no unit and is not used; (3) confirm from the TPS cube manual which control sets pH 4 - the source says "the same as pH 7"; (4) set the acceptable pH electrode slope range; (5) confirm the Mt. Morgan records for DO results and pH calibration - the Martabe Daily Task Checklist (DOC-FRM-00052-EN) and form DOC-4-MET-PMC-DFR-00142-EN are source names; (6) conductivity standards are not held - conductivity meters cannot be calibrated until they are.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1567,49 +1807,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Register seri 206 Met Lab Operations and Safety (11 dokumen dalam format Heritage).</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Register seri 206 Met Lab Operations and Safety (13 dokumen dalam format Heritage).</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx, ditimpa oleh keputusan review bila ada. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Jumlah step dan halaman dihitung dari render dokumen (LibreOffice); halaman bisa sedikit berbeda di Microsoft Word.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Status isi: Final = tanpa tambahan Martabe terbuka; DRAFT FOR REVIEW = ada tambahan Martabe yang menunggu JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Sheet "Draft dan open items" memuat paragraf draft, catatan, temuan safety-critical, dan open items di Description of work.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Referensi register: HM-MMM-WHS-REG-XXX-R00-SWI-SWMS, tab SWI-MET.</t>
         </is>

</xml_diff>